<commit_message>
Fix Vietnamese translation flow
</commit_message>
<xml_diff>
--- a/04-Bieu-Mau/02-FRM-200/FRM-202_Contract_Review_Checklist.xlsx
+++ b/04-Bieu-Mau/02-FRM-200/FRM-202_Contract_Review_Checklist.xlsx
@@ -8,6 +8,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_IMPORT" sheetId="3" state="veryHidden" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ACTIONS" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REF_LINKS" sheetId="5" state="veryHidden" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_REVHIST" sheetId="6" state="hidden" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="VAL_RESULT_CORE">'_LISTS'!$A$2:$A$5</definedName>
@@ -524,7 +525,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="57">
+  <fills count="64">
     <fill>
       <patternFill/>
     </fill>
@@ -806,8 +807,50 @@
         <fgColor rgb="00F7F9FC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F1F5F9"/>
+        <bgColor rgb="00F1F5F9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D7F0E2"/>
+        <bgColor rgb="00D7F0E2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+        <bgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8FAFC"/>
+        <bgColor rgb="00F8FAFC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF3C4"/>
+        <bgColor rgb="00FFF3C4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F0D7E8"/>
+        <bgColor rgb="00F0D7E8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00005A9E"/>
+        <bgColor rgb="00005A9E"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="290">
+  <borders count="292">
     <border>
       <left/>
       <right/>
@@ -3942,6 +3985,34 @@
       <right/>
       <top style="thin">
         <color rgb="00E2E8F0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="000078D4"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="000078D4"/>
+      </left>
+      <right style="thin">
+        <color rgb="00E2E8F0"/>
+      </right>
+      <top style="thin">
+        <color rgb="000078D4"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="000078D4"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00E2E8F0"/>
+      </left>
+      <right style="thin">
+        <color rgb="00E2E8F0"/>
+      </right>
+      <top style="thin">
+        <color rgb="000078D4"/>
       </top>
       <bottom style="thin">
         <color rgb="000078D4"/>
@@ -3951,7 +4022,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="398">
+  <cellXfs count="415">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -4892,10 +4963,101 @@
     <xf numFmtId="0" fontId="17" fillId="7" borderId="130" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="2"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="57" borderId="290" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="58" borderId="291" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="59" borderId="291" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="57" borderId="291" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="59" borderId="291" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="59" borderId="285" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="60" borderId="291" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="61" borderId="291" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="62" borderId="291" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="57" borderId="290" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="59" borderId="291" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="57" borderId="291" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="59" borderId="285" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="57" borderId="291" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="57" borderId="285" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="63" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0"/>
   </cellStyles>
+  <dxfs count="4">
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="00CC0000"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFCCCC"/>
+          <bgColor rgb="00FFCCCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFF3C4"/>
+          <bgColor rgb="00FFF3C4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00D7F0E2"/>
+          <bgColor rgb="00D7F0E2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00DBEAFE"/>
+          <bgColor rgb="00DBEAFE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -4978,7 +5140,7 @@
         <t>Linked SOP/WI/ANNEX: SOP-201 | WI-201/WI-202/WI-203/WI-207 | ANNEX-QMS-020 + ANNEX-QMS-008</t>
       </text>
     </comment>
-    <comment ref="A47" authorId="0" shapeId="0">
+    <comment ref="A54" authorId="0" shapeId="0">
       <text>
         <t>Upstream: FRM-201 / FRM-301 / FRM-303 / customer PO evidence. Downstream: FRM-204 / FRM-209 / FRM-501 / FRM-519.</t>
       </text>
@@ -5299,7 +5461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr autoPageBreaks="0" fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AN47"/>
+  <dimension ref="A1:AN54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.329999923706055" customWidth="1" min="1" max="1"/>
@@ -5412,7 +5574,7 @@
       <c r="AH2" s="278" t="n"/>
       <c r="AI2" s="279" t="inlineStr">
         <is>
-          <t>V0</t>
+          <t>V1</t>
         </is>
       </c>
       <c r="AJ2" s="277" t="n"/>
@@ -5455,7 +5617,7 @@
       <c r="AH3" s="278" t="n"/>
       <c r="AI3" s="279" t="inlineStr">
         <is>
-          <t>YYYY-MM-DD</t>
+          <t>2026-03-22</t>
         </is>
       </c>
       <c r="AJ3" s="277" t="n"/>
@@ -5933,7 +6095,7 @@
       <c r="Z15" s="271" t="n"/>
       <c r="AA15" s="272" t="n"/>
       <c r="AB15" s="294">
-        <f>IF(COUNTA(AF22:AF31)=0,"",IF(COUNTIF(AF22:AF31,"FAIL")+COUNTIF(AF22:AF31,"HOLD")&gt;0,"HOLD",IF(COUNTIF(AF22:AF31,"PASS")=COUNTA(AF22:AF31),"APPROVED","CONDITIONAL")))</f>
+        <f>IF(COUNTA(AF22:AF36)=0,"",IF(COUNTIF(AF22:AF36,"FAIL")+COUNTIF(AF22:AF36,"HOLD")&gt;0,"HOLD",IF(COUNTIF(AF22:AF36,"PASS")=COUNTA(AF22:AF36),"APPROVED","REVIEW")))</f>
         <v/>
       </c>
       <c r="AC15" s="271" t="n"/>
@@ -6086,7 +6248,7 @@
       <c r="Z18" s="283" t="n"/>
       <c r="AA18" s="285" t="n"/>
       <c r="AB18" s="286">
-        <f>IF(COUNTA(AF22:AF31)=0,"",IF(COUNTIF(AF22:AF31,"FAIL")+COUNTIF(AF22:AF31,"HOLD")&gt;0,"OPEN","CLOSED"))</f>
+        <f>IF(COUNTA(AF22:AF36)=0,"",IF(COUNTIF(AF22:AF36,"FAIL")+COUNTIF(AF22:AF36,"HOLD")&gt;0,"OPEN","CLOSED"))</f>
         <v/>
       </c>
       <c r="AC18" s="283" t="n"/>
@@ -6781,608 +6943,752 @@
       <c r="AM31" s="308" t="n"/>
       <c r="AN31" s="333" t="n"/>
     </row>
-    <row r="32" ht="4" customHeight="1">
-      <c r="A32" s="25" t="n"/>
-    </row>
-    <row r="33" ht="17" customHeight="1">
-      <c r="A33" s="288" t="inlineStr">
+    <row r="32" ht="20" customHeight="1">
+      <c r="A32" s="398" t="n">
+        <v>11</v>
+      </c>
+      <c r="C32" s="399" t="inlineStr">
+        <is>
+          <t>TEC</t>
+        </is>
+      </c>
+      <c r="F32" s="400" t="inlineStr">
+        <is>
+          <t>CNC program revision matches released drawing revision.</t>
+        </is>
+      </c>
+      <c r="T32" s="401" t="inlineStr">
+        <is>
+          <t>Program rev, drawing rev, setup sheet rev all align.</t>
+        </is>
+      </c>
+      <c r="AF32" s="402" t="n"/>
+      <c r="AJ32" s="402" t="n"/>
+      <c r="AM32" s="403" t="n"/>
+    </row>
+    <row r="33" ht="20" customHeight="1">
+      <c r="A33" s="398" t="n">
+        <v>12</v>
+      </c>
+      <c r="C33" s="399" t="inlineStr">
+        <is>
+          <t>TEC</t>
+        </is>
+      </c>
+      <c r="F33" s="404" t="inlineStr">
+        <is>
+          <t>Tight-tolerance features identified (&lt; 0.025 mm).</t>
+        </is>
+      </c>
+      <c r="T33" s="401" t="inlineStr">
+        <is>
+          <t>Feature count flagged; measurement method confirmed.</t>
+        </is>
+      </c>
+      <c r="AF33" s="402" t="n"/>
+      <c r="AJ33" s="402" t="n"/>
+      <c r="AM33" s="403" t="n"/>
+    </row>
+    <row r="34" ht="20" customHeight="1">
+      <c r="A34" s="398" t="n">
+        <v>13</v>
+      </c>
+      <c r="C34" s="405" t="inlineStr">
+        <is>
+          <t>QUA</t>
+        </is>
+      </c>
+      <c r="F34" s="400" t="inlineStr">
+        <is>
+          <t>Semiconductor cleanliness class confirmed.</t>
+        </is>
+      </c>
+      <c r="T34" s="401" t="inlineStr">
+        <is>
+          <t>Clean-room / clean-pack / vacuum-bag level specified or NA.</t>
+        </is>
+      </c>
+      <c r="AF34" s="402" t="n"/>
+      <c r="AJ34" s="402" t="n"/>
+      <c r="AM34" s="403" t="n"/>
+    </row>
+    <row r="35" ht="20" customHeight="1">
+      <c r="A35" s="398" t="n">
+        <v>14</v>
+      </c>
+      <c r="C35" s="405" t="inlineStr">
+        <is>
+          <t>QUA</t>
+        </is>
+      </c>
+      <c r="F35" s="404" t="inlineStr">
+        <is>
+          <t>Material cert / CoC / test-report requirement specified.</t>
+        </is>
+      </c>
+      <c r="T35" s="401" t="inlineStr">
+        <is>
+          <t>Cert type, mill cert, RoHS, REACH, or conflict minerals.</t>
+        </is>
+      </c>
+      <c r="AF35" s="402" t="n"/>
+      <c r="AJ35" s="402" t="n"/>
+      <c r="AM35" s="403" t="n"/>
+    </row>
+    <row r="36" ht="20" customHeight="1">
+      <c r="A36" s="398" t="n">
+        <v>15</v>
+      </c>
+      <c r="C36" s="406" t="inlineStr">
+        <is>
+          <t>CAP</t>
+        </is>
+      </c>
+      <c r="F36" s="400" t="inlineStr">
+        <is>
+          <t>Outsource processes (HT/plate/anod) confirmed with lead time.</t>
+        </is>
+      </c>
+      <c r="T36" s="401" t="inlineStr">
+        <is>
+          <t>Supplier approved, lead time fits delivery promise.</t>
+        </is>
+      </c>
+      <c r="AF36" s="402" t="n"/>
+      <c r="AJ36" s="402" t="n"/>
+      <c r="AM36" s="403" t="n"/>
+    </row>
+    <row r="37" ht="20" customHeight="1">
+      <c r="A37" s="407" t="inlineStr">
+        <is>
+          <t>Linked FRM-203 Job #</t>
+        </is>
+      </c>
+      <c r="H37" s="408" t="n"/>
+      <c r="U37" s="409" t="inlineStr">
+        <is>
+          <t>Linked FRM-204 Kickoff #</t>
+        </is>
+      </c>
+      <c r="AB37" s="410" t="n"/>
+    </row>
+    <row r="38" ht="20" customHeight="1">
+      <c r="A38" s="407" t="inlineStr">
+        <is>
+          <t>Ref: SOP-201 / WI-201~203</t>
+        </is>
+      </c>
+      <c r="H38" s="411" t="inlineStr">
+        <is>
+          <t>SOP-201 (RFQ, Contract Review, Order Kickoff)</t>
+        </is>
+      </c>
+      <c r="U38" s="409" t="inlineStr">
+        <is>
+          <t>Retain: 10 years</t>
+        </is>
+      </c>
+      <c r="AB38" s="412" t="inlineStr">
+        <is>
+          <t>Per QMS retention schedule</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="20" customHeight="1">
+      <c r="A39" s="25" t="n"/>
+    </row>
+    <row r="40" ht="4" customHeight="1">
+      <c r="A40" s="288" t="inlineStr">
         <is>
           <t>4.  OPEN CONDITIONS / ACTION TRACKER</t>
         </is>
       </c>
-      <c r="B33" s="289" t="n"/>
-      <c r="C33" s="289" t="n"/>
-      <c r="D33" s="289" t="n"/>
-      <c r="E33" s="289" t="n"/>
-      <c r="F33" s="289" t="n"/>
-      <c r="G33" s="289" t="n"/>
-      <c r="H33" s="289" t="n"/>
-      <c r="I33" s="289" t="n"/>
-      <c r="J33" s="289" t="n"/>
-      <c r="K33" s="289" t="n"/>
-      <c r="L33" s="289" t="n"/>
-      <c r="M33" s="289" t="n"/>
-      <c r="N33" s="289" t="n"/>
-      <c r="O33" s="289" t="n"/>
-      <c r="P33" s="289" t="n"/>
-      <c r="Q33" s="289" t="n"/>
-      <c r="R33" s="289" t="n"/>
-      <c r="S33" s="289" t="n"/>
-      <c r="T33" s="289" t="n"/>
-      <c r="U33" s="289" t="n"/>
-      <c r="V33" s="289" t="n"/>
-      <c r="W33" s="289" t="n"/>
-      <c r="X33" s="289" t="n"/>
-      <c r="Y33" s="289" t="n"/>
-      <c r="Z33" s="289" t="n"/>
-      <c r="AA33" s="289" t="n"/>
-      <c r="AB33" s="289" t="n"/>
-      <c r="AC33" s="289" t="n"/>
-      <c r="AD33" s="289" t="n"/>
-      <c r="AE33" s="289" t="n"/>
-      <c r="AF33" s="289" t="n"/>
-      <c r="AG33" s="289" t="n"/>
-      <c r="AH33" s="289" t="n"/>
-      <c r="AI33" s="289" t="n"/>
-      <c r="AJ33" s="289" t="n"/>
-      <c r="AK33" s="289" t="n"/>
-      <c r="AL33" s="289" t="n"/>
-      <c r="AM33" s="289" t="n"/>
-      <c r="AN33" s="290" t="n"/>
-    </row>
-    <row r="34" ht="17" customHeight="1">
-      <c r="A34" s="301" t="inlineStr">
+      <c r="B40" s="289" t="n"/>
+      <c r="C40" s="289" t="n"/>
+      <c r="D40" s="289" t="n"/>
+      <c r="E40" s="289" t="n"/>
+      <c r="F40" s="289" t="n"/>
+      <c r="G40" s="289" t="n"/>
+      <c r="H40" s="289" t="n"/>
+      <c r="I40" s="289" t="n"/>
+      <c r="J40" s="289" t="n"/>
+      <c r="K40" s="289" t="n"/>
+      <c r="L40" s="289" t="n"/>
+      <c r="M40" s="289" t="n"/>
+      <c r="N40" s="289" t="n"/>
+      <c r="O40" s="289" t="n"/>
+      <c r="P40" s="289" t="n"/>
+      <c r="Q40" s="289" t="n"/>
+      <c r="R40" s="289" t="n"/>
+      <c r="S40" s="289" t="n"/>
+      <c r="T40" s="289" t="n"/>
+      <c r="U40" s="289" t="n"/>
+      <c r="V40" s="289" t="n"/>
+      <c r="W40" s="289" t="n"/>
+      <c r="X40" s="289" t="n"/>
+      <c r="Y40" s="289" t="n"/>
+      <c r="Z40" s="289" t="n"/>
+      <c r="AA40" s="289" t="n"/>
+      <c r="AB40" s="289" t="n"/>
+      <c r="AC40" s="289" t="n"/>
+      <c r="AD40" s="289" t="n"/>
+      <c r="AE40" s="289" t="n"/>
+      <c r="AF40" s="289" t="n"/>
+      <c r="AG40" s="289" t="n"/>
+      <c r="AH40" s="289" t="n"/>
+      <c r="AI40" s="289" t="n"/>
+      <c r="AJ40" s="289" t="n"/>
+      <c r="AK40" s="289" t="n"/>
+      <c r="AL40" s="289" t="n"/>
+      <c r="AM40" s="289" t="n"/>
+      <c r="AN40" s="290" t="n"/>
+    </row>
+    <row r="41" ht="17" customHeight="1">
+      <c r="A41" s="301" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B34" s="272" t="n"/>
-      <c r="C34" s="302" t="inlineStr">
+      <c r="B41" s="272" t="n"/>
+      <c r="C41" s="302" t="inlineStr">
         <is>
           <t>Issue / Open Condition</t>
         </is>
       </c>
-      <c r="D34" s="271" t="n"/>
-      <c r="E34" s="271" t="n"/>
-      <c r="F34" s="271" t="n"/>
-      <c r="G34" s="271" t="n"/>
-      <c r="H34" s="271" t="n"/>
-      <c r="I34" s="271" t="n"/>
-      <c r="J34" s="271" t="n"/>
-      <c r="K34" s="271" t="n"/>
-      <c r="L34" s="272" t="n"/>
-      <c r="M34" s="302" t="inlineStr">
+      <c r="D41" s="271" t="n"/>
+      <c r="E41" s="271" t="n"/>
+      <c r="F41" s="271" t="n"/>
+      <c r="G41" s="271" t="n"/>
+      <c r="H41" s="271" t="n"/>
+      <c r="I41" s="271" t="n"/>
+      <c r="J41" s="271" t="n"/>
+      <c r="K41" s="271" t="n"/>
+      <c r="L41" s="272" t="n"/>
+      <c r="M41" s="302" t="inlineStr">
         <is>
           <t>Required Action</t>
         </is>
       </c>
-      <c r="N34" s="271" t="n"/>
-      <c r="O34" s="271" t="n"/>
-      <c r="P34" s="271" t="n"/>
-      <c r="Q34" s="271" t="n"/>
-      <c r="R34" s="271" t="n"/>
-      <c r="S34" s="271" t="n"/>
-      <c r="T34" s="271" t="n"/>
-      <c r="U34" s="271" t="n"/>
-      <c r="V34" s="271" t="n"/>
-      <c r="W34" s="271" t="n"/>
-      <c r="X34" s="272" t="n"/>
-      <c r="Y34" s="302" t="inlineStr">
+      <c r="N41" s="271" t="n"/>
+      <c r="O41" s="271" t="n"/>
+      <c r="P41" s="271" t="n"/>
+      <c r="Q41" s="271" t="n"/>
+      <c r="R41" s="271" t="n"/>
+      <c r="S41" s="271" t="n"/>
+      <c r="T41" s="271" t="n"/>
+      <c r="U41" s="271" t="n"/>
+      <c r="V41" s="271" t="n"/>
+      <c r="W41" s="271" t="n"/>
+      <c r="X41" s="272" t="n"/>
+      <c r="Y41" s="302" t="inlineStr">
         <is>
           <t>Owner</t>
         </is>
       </c>
-      <c r="Z34" s="271" t="n"/>
-      <c r="AA34" s="271" t="n"/>
-      <c r="AB34" s="271" t="n"/>
-      <c r="AC34" s="272" t="n"/>
-      <c r="AD34" s="302" t="inlineStr">
+      <c r="Z41" s="271" t="n"/>
+      <c r="AA41" s="271" t="n"/>
+      <c r="AB41" s="271" t="n"/>
+      <c r="AC41" s="272" t="n"/>
+      <c r="AD41" s="302" t="inlineStr">
         <is>
           <t>Due Date</t>
         </is>
       </c>
-      <c r="AE34" s="271" t="n"/>
-      <c r="AF34" s="271" t="n"/>
-      <c r="AG34" s="271" t="n"/>
-      <c r="AH34" s="272" t="n"/>
-      <c r="AI34" s="302" t="inlineStr">
+      <c r="AE41" s="271" t="n"/>
+      <c r="AF41" s="271" t="n"/>
+      <c r="AG41" s="271" t="n"/>
+      <c r="AH41" s="272" t="n"/>
+      <c r="AI41" s="302" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="AJ34" s="271" t="n"/>
-      <c r="AK34" s="272" t="n"/>
-      <c r="AL34" s="303" t="inlineStr">
+      <c r="AJ41" s="271" t="n"/>
+      <c r="AK41" s="272" t="n"/>
+      <c r="AL41" s="303" t="inlineStr">
         <is>
           <t>Verified by</t>
         </is>
       </c>
-      <c r="AM34" s="271" t="n"/>
-      <c r="AN34" s="274" t="n"/>
-    </row>
-    <row r="35" ht="20" customHeight="1">
-      <c r="A35" s="318" t="n">
+      <c r="AM41" s="271" t="n"/>
+      <c r="AN41" s="274" t="n"/>
+    </row>
+    <row r="42" ht="17" customHeight="1">
+      <c r="A42" s="318" t="n">
         <v>1</v>
       </c>
-      <c r="B35" s="278" t="n"/>
-      <c r="C35" s="308" t="n"/>
-      <c r="D35" s="334" t="n"/>
-      <c r="E35" s="334" t="n"/>
-      <c r="F35" s="334" t="n"/>
-      <c r="G35" s="334" t="n"/>
-      <c r="H35" s="334" t="n"/>
-      <c r="I35" s="334" t="n"/>
-      <c r="J35" s="334" t="n"/>
-      <c r="K35" s="334" t="n"/>
-      <c r="L35" s="333" t="n"/>
-      <c r="M35" s="308" t="n"/>
-      <c r="N35" s="334" t="n"/>
-      <c r="O35" s="334" t="n"/>
-      <c r="P35" s="334" t="n"/>
-      <c r="Q35" s="334" t="n"/>
-      <c r="R35" s="334" t="n"/>
-      <c r="S35" s="334" t="n"/>
-      <c r="T35" s="334" t="n"/>
-      <c r="U35" s="334" t="n"/>
-      <c r="V35" s="334" t="n"/>
-      <c r="W35" s="334" t="n"/>
-      <c r="X35" s="333" t="n"/>
-      <c r="Y35" s="308" t="n"/>
-      <c r="Z35" s="334" t="n"/>
-      <c r="AA35" s="334" t="n"/>
-      <c r="AB35" s="334" t="n"/>
-      <c r="AC35" s="333" t="n"/>
-      <c r="AD35" s="308" t="n"/>
-      <c r="AE35" s="334" t="n"/>
-      <c r="AF35" s="334" t="n"/>
-      <c r="AG35" s="334" t="n"/>
-      <c r="AH35" s="333" t="n"/>
-      <c r="AI35" s="308" t="n"/>
-      <c r="AJ35" s="334" t="n"/>
-      <c r="AK35" s="333" t="n"/>
-      <c r="AL35" s="308" t="n"/>
-      <c r="AM35" s="334" t="n"/>
-      <c r="AN35" s="333" t="n"/>
-    </row>
-    <row r="36" ht="20" customHeight="1">
-      <c r="A36" s="318" t="n">
+      <c r="B42" s="278" t="n"/>
+      <c r="C42" s="308" t="n"/>
+      <c r="D42" s="334" t="n"/>
+      <c r="E42" s="334" t="n"/>
+      <c r="F42" s="334" t="n"/>
+      <c r="G42" s="334" t="n"/>
+      <c r="H42" s="334" t="n"/>
+      <c r="I42" s="334" t="n"/>
+      <c r="J42" s="334" t="n"/>
+      <c r="K42" s="334" t="n"/>
+      <c r="L42" s="333" t="n"/>
+      <c r="M42" s="308" t="n"/>
+      <c r="N42" s="334" t="n"/>
+      <c r="O42" s="334" t="n"/>
+      <c r="P42" s="334" t="n"/>
+      <c r="Q42" s="334" t="n"/>
+      <c r="R42" s="334" t="n"/>
+      <c r="S42" s="334" t="n"/>
+      <c r="T42" s="334" t="n"/>
+      <c r="U42" s="334" t="n"/>
+      <c r="V42" s="334" t="n"/>
+      <c r="W42" s="334" t="n"/>
+      <c r="X42" s="333" t="n"/>
+      <c r="Y42" s="308" t="n"/>
+      <c r="Z42" s="334" t="n"/>
+      <c r="AA42" s="334" t="n"/>
+      <c r="AB42" s="334" t="n"/>
+      <c r="AC42" s="333" t="n"/>
+      <c r="AD42" s="308" t="n"/>
+      <c r="AE42" s="334" t="n"/>
+      <c r="AF42" s="334" t="n"/>
+      <c r="AG42" s="334" t="n"/>
+      <c r="AH42" s="333" t="n"/>
+      <c r="AI42" s="308" t="n"/>
+      <c r="AJ42" s="334" t="n"/>
+      <c r="AK42" s="333" t="n"/>
+      <c r="AL42" s="308" t="n"/>
+      <c r="AM42" s="334" t="n"/>
+      <c r="AN42" s="333" t="n"/>
+    </row>
+    <row r="43" ht="26" customHeight="1">
+      <c r="A43" s="318" t="n">
         <v>2</v>
       </c>
-      <c r="B36" s="278" t="n"/>
-      <c r="C36" s="308" t="n"/>
-      <c r="D36" s="334" t="n"/>
-      <c r="E36" s="334" t="n"/>
-      <c r="F36" s="334" t="n"/>
-      <c r="G36" s="334" t="n"/>
-      <c r="H36" s="334" t="n"/>
-      <c r="I36" s="334" t="n"/>
-      <c r="J36" s="334" t="n"/>
-      <c r="K36" s="334" t="n"/>
-      <c r="L36" s="333" t="n"/>
-      <c r="M36" s="308" t="n"/>
-      <c r="N36" s="334" t="n"/>
-      <c r="O36" s="334" t="n"/>
-      <c r="P36" s="334" t="n"/>
-      <c r="Q36" s="334" t="n"/>
-      <c r="R36" s="334" t="n"/>
-      <c r="S36" s="334" t="n"/>
-      <c r="T36" s="334" t="n"/>
-      <c r="U36" s="334" t="n"/>
-      <c r="V36" s="334" t="n"/>
-      <c r="W36" s="334" t="n"/>
-      <c r="X36" s="333" t="n"/>
-      <c r="Y36" s="308" t="n"/>
-      <c r="Z36" s="334" t="n"/>
-      <c r="AA36" s="334" t="n"/>
-      <c r="AB36" s="334" t="n"/>
-      <c r="AC36" s="333" t="n"/>
-      <c r="AD36" s="308" t="n"/>
-      <c r="AE36" s="334" t="n"/>
-      <c r="AF36" s="334" t="n"/>
-      <c r="AG36" s="334" t="n"/>
-      <c r="AH36" s="333" t="n"/>
-      <c r="AI36" s="308" t="n"/>
-      <c r="AJ36" s="334" t="n"/>
-      <c r="AK36" s="333" t="n"/>
-      <c r="AL36" s="308" t="n"/>
-      <c r="AM36" s="334" t="n"/>
-      <c r="AN36" s="333" t="n"/>
-    </row>
-    <row r="37" ht="20" customHeight="1">
-      <c r="A37" s="318" t="n">
+      <c r="B43" s="278" t="n"/>
+      <c r="C43" s="308" t="n"/>
+      <c r="D43" s="334" t="n"/>
+      <c r="E43" s="334" t="n"/>
+      <c r="F43" s="334" t="n"/>
+      <c r="G43" s="334" t="n"/>
+      <c r="H43" s="334" t="n"/>
+      <c r="I43" s="334" t="n"/>
+      <c r="J43" s="334" t="n"/>
+      <c r="K43" s="334" t="n"/>
+      <c r="L43" s="333" t="n"/>
+      <c r="M43" s="308" t="n"/>
+      <c r="N43" s="334" t="n"/>
+      <c r="O43" s="334" t="n"/>
+      <c r="P43" s="334" t="n"/>
+      <c r="Q43" s="334" t="n"/>
+      <c r="R43" s="334" t="n"/>
+      <c r="S43" s="334" t="n"/>
+      <c r="T43" s="334" t="n"/>
+      <c r="U43" s="334" t="n"/>
+      <c r="V43" s="334" t="n"/>
+      <c r="W43" s="334" t="n"/>
+      <c r="X43" s="333" t="n"/>
+      <c r="Y43" s="308" t="n"/>
+      <c r="Z43" s="334" t="n"/>
+      <c r="AA43" s="334" t="n"/>
+      <c r="AB43" s="334" t="n"/>
+      <c r="AC43" s="333" t="n"/>
+      <c r="AD43" s="308" t="n"/>
+      <c r="AE43" s="334" t="n"/>
+      <c r="AF43" s="334" t="n"/>
+      <c r="AG43" s="334" t="n"/>
+      <c r="AH43" s="333" t="n"/>
+      <c r="AI43" s="308" t="n"/>
+      <c r="AJ43" s="334" t="n"/>
+      <c r="AK43" s="333" t="n"/>
+      <c r="AL43" s="308" t="n"/>
+      <c r="AM43" s="334" t="n"/>
+      <c r="AN43" s="333" t="n"/>
+    </row>
+    <row r="44" ht="26" customHeight="1">
+      <c r="A44" s="318" t="n">
         <v>3</v>
       </c>
-      <c r="B37" s="278" t="n"/>
-      <c r="C37" s="308" t="n"/>
-      <c r="D37" s="334" t="n"/>
-      <c r="E37" s="334" t="n"/>
-      <c r="F37" s="334" t="n"/>
-      <c r="G37" s="334" t="n"/>
-      <c r="H37" s="334" t="n"/>
-      <c r="I37" s="334" t="n"/>
-      <c r="J37" s="334" t="n"/>
-      <c r="K37" s="334" t="n"/>
-      <c r="L37" s="333" t="n"/>
-      <c r="M37" s="308" t="n"/>
-      <c r="N37" s="334" t="n"/>
-      <c r="O37" s="334" t="n"/>
-      <c r="P37" s="334" t="n"/>
-      <c r="Q37" s="334" t="n"/>
-      <c r="R37" s="334" t="n"/>
-      <c r="S37" s="334" t="n"/>
-      <c r="T37" s="334" t="n"/>
-      <c r="U37" s="334" t="n"/>
-      <c r="V37" s="334" t="n"/>
-      <c r="W37" s="334" t="n"/>
-      <c r="X37" s="333" t="n"/>
-      <c r="Y37" s="308" t="n"/>
-      <c r="Z37" s="334" t="n"/>
-      <c r="AA37" s="334" t="n"/>
-      <c r="AB37" s="334" t="n"/>
-      <c r="AC37" s="333" t="n"/>
-      <c r="AD37" s="308" t="n"/>
-      <c r="AE37" s="334" t="n"/>
-      <c r="AF37" s="334" t="n"/>
-      <c r="AG37" s="334" t="n"/>
-      <c r="AH37" s="333" t="n"/>
-      <c r="AI37" s="308" t="n"/>
-      <c r="AJ37" s="334" t="n"/>
-      <c r="AK37" s="333" t="n"/>
-      <c r="AL37" s="308" t="n"/>
-      <c r="AM37" s="334" t="n"/>
-      <c r="AN37" s="333" t="n"/>
-    </row>
-    <row r="38" ht="20" customHeight="1">
-      <c r="A38" s="318" t="n">
+      <c r="B44" s="278" t="n"/>
+      <c r="C44" s="308" t="n"/>
+      <c r="D44" s="334" t="n"/>
+      <c r="E44" s="334" t="n"/>
+      <c r="F44" s="334" t="n"/>
+      <c r="G44" s="334" t="n"/>
+      <c r="H44" s="334" t="n"/>
+      <c r="I44" s="334" t="n"/>
+      <c r="J44" s="334" t="n"/>
+      <c r="K44" s="334" t="n"/>
+      <c r="L44" s="333" t="n"/>
+      <c r="M44" s="308" t="n"/>
+      <c r="N44" s="334" t="n"/>
+      <c r="O44" s="334" t="n"/>
+      <c r="P44" s="334" t="n"/>
+      <c r="Q44" s="334" t="n"/>
+      <c r="R44" s="334" t="n"/>
+      <c r="S44" s="334" t="n"/>
+      <c r="T44" s="334" t="n"/>
+      <c r="U44" s="334" t="n"/>
+      <c r="V44" s="334" t="n"/>
+      <c r="W44" s="334" t="n"/>
+      <c r="X44" s="333" t="n"/>
+      <c r="Y44" s="308" t="n"/>
+      <c r="Z44" s="334" t="n"/>
+      <c r="AA44" s="334" t="n"/>
+      <c r="AB44" s="334" t="n"/>
+      <c r="AC44" s="333" t="n"/>
+      <c r="AD44" s="308" t="n"/>
+      <c r="AE44" s="334" t="n"/>
+      <c r="AF44" s="334" t="n"/>
+      <c r="AG44" s="334" t="n"/>
+      <c r="AH44" s="333" t="n"/>
+      <c r="AI44" s="308" t="n"/>
+      <c r="AJ44" s="334" t="n"/>
+      <c r="AK44" s="333" t="n"/>
+      <c r="AL44" s="308" t="n"/>
+      <c r="AM44" s="334" t="n"/>
+      <c r="AN44" s="333" t="n"/>
+    </row>
+    <row r="45" ht="26" customHeight="1">
+      <c r="A45" s="318" t="n">
         <v>4</v>
       </c>
-      <c r="B38" s="278" t="n"/>
-      <c r="C38" s="308" t="n"/>
-      <c r="D38" s="334" t="n"/>
-      <c r="E38" s="334" t="n"/>
-      <c r="F38" s="334" t="n"/>
-      <c r="G38" s="334" t="n"/>
-      <c r="H38" s="334" t="n"/>
-      <c r="I38" s="334" t="n"/>
-      <c r="J38" s="334" t="n"/>
-      <c r="K38" s="334" t="n"/>
-      <c r="L38" s="333" t="n"/>
-      <c r="M38" s="308" t="n"/>
-      <c r="N38" s="334" t="n"/>
-      <c r="O38" s="334" t="n"/>
-      <c r="P38" s="334" t="n"/>
-      <c r="Q38" s="334" t="n"/>
-      <c r="R38" s="334" t="n"/>
-      <c r="S38" s="334" t="n"/>
-      <c r="T38" s="334" t="n"/>
-      <c r="U38" s="334" t="n"/>
-      <c r="V38" s="334" t="n"/>
-      <c r="W38" s="334" t="n"/>
-      <c r="X38" s="333" t="n"/>
-      <c r="Y38" s="308" t="n"/>
-      <c r="Z38" s="334" t="n"/>
-      <c r="AA38" s="334" t="n"/>
-      <c r="AB38" s="334" t="n"/>
-      <c r="AC38" s="333" t="n"/>
-      <c r="AD38" s="308" t="n"/>
-      <c r="AE38" s="334" t="n"/>
-      <c r="AF38" s="334" t="n"/>
-      <c r="AG38" s="334" t="n"/>
-      <c r="AH38" s="333" t="n"/>
-      <c r="AI38" s="308" t="n"/>
-      <c r="AJ38" s="334" t="n"/>
-      <c r="AK38" s="333" t="n"/>
-      <c r="AL38" s="308" t="n"/>
-      <c r="AM38" s="334" t="n"/>
-      <c r="AN38" s="333" t="n"/>
-    </row>
-    <row r="39" ht="20" customHeight="1">
-      <c r="A39" s="319" t="n">
+      <c r="B45" s="278" t="n"/>
+      <c r="C45" s="308" t="n"/>
+      <c r="D45" s="334" t="n"/>
+      <c r="E45" s="334" t="n"/>
+      <c r="F45" s="334" t="n"/>
+      <c r="G45" s="334" t="n"/>
+      <c r="H45" s="334" t="n"/>
+      <c r="I45" s="334" t="n"/>
+      <c r="J45" s="334" t="n"/>
+      <c r="K45" s="334" t="n"/>
+      <c r="L45" s="333" t="n"/>
+      <c r="M45" s="308" t="n"/>
+      <c r="N45" s="334" t="n"/>
+      <c r="O45" s="334" t="n"/>
+      <c r="P45" s="334" t="n"/>
+      <c r="Q45" s="334" t="n"/>
+      <c r="R45" s="334" t="n"/>
+      <c r="S45" s="334" t="n"/>
+      <c r="T45" s="334" t="n"/>
+      <c r="U45" s="334" t="n"/>
+      <c r="V45" s="334" t="n"/>
+      <c r="W45" s="334" t="n"/>
+      <c r="X45" s="333" t="n"/>
+      <c r="Y45" s="308" t="n"/>
+      <c r="Z45" s="334" t="n"/>
+      <c r="AA45" s="334" t="n"/>
+      <c r="AB45" s="334" t="n"/>
+      <c r="AC45" s="333" t="n"/>
+      <c r="AD45" s="308" t="n"/>
+      <c r="AE45" s="334" t="n"/>
+      <c r="AF45" s="334" t="n"/>
+      <c r="AG45" s="334" t="n"/>
+      <c r="AH45" s="333" t="n"/>
+      <c r="AI45" s="308" t="n"/>
+      <c r="AJ45" s="334" t="n"/>
+      <c r="AK45" s="333" t="n"/>
+      <c r="AL45" s="308" t="n"/>
+      <c r="AM45" s="334" t="n"/>
+      <c r="AN45" s="333" t="n"/>
+    </row>
+    <row r="46" ht="4" customHeight="1">
+      <c r="A46" s="319" t="n">
         <v>5</v>
       </c>
-      <c r="B39" s="285" t="n"/>
-      <c r="C39" s="308" t="n"/>
-      <c r="D39" s="334" t="n"/>
-      <c r="E39" s="334" t="n"/>
-      <c r="F39" s="334" t="n"/>
-      <c r="G39" s="334" t="n"/>
-      <c r="H39" s="334" t="n"/>
-      <c r="I39" s="334" t="n"/>
-      <c r="J39" s="334" t="n"/>
-      <c r="K39" s="334" t="n"/>
-      <c r="L39" s="333" t="n"/>
-      <c r="M39" s="308" t="n"/>
-      <c r="N39" s="334" t="n"/>
-      <c r="O39" s="334" t="n"/>
-      <c r="P39" s="334" t="n"/>
-      <c r="Q39" s="334" t="n"/>
-      <c r="R39" s="334" t="n"/>
-      <c r="S39" s="334" t="n"/>
-      <c r="T39" s="334" t="n"/>
-      <c r="U39" s="334" t="n"/>
-      <c r="V39" s="334" t="n"/>
-      <c r="W39" s="334" t="n"/>
-      <c r="X39" s="333" t="n"/>
-      <c r="Y39" s="308" t="n"/>
-      <c r="Z39" s="334" t="n"/>
-      <c r="AA39" s="334" t="n"/>
-      <c r="AB39" s="334" t="n"/>
-      <c r="AC39" s="333" t="n"/>
-      <c r="AD39" s="308" t="n"/>
-      <c r="AE39" s="334" t="n"/>
-      <c r="AF39" s="334" t="n"/>
-      <c r="AG39" s="334" t="n"/>
-      <c r="AH39" s="333" t="n"/>
-      <c r="AI39" s="308" t="n"/>
-      <c r="AJ39" s="334" t="n"/>
-      <c r="AK39" s="333" t="n"/>
-      <c r="AL39" s="308" t="n"/>
-      <c r="AM39" s="334" t="n"/>
-      <c r="AN39" s="333" t="n"/>
-    </row>
-    <row r="40" ht="4" customHeight="1">
-      <c r="A40" s="25" t="n"/>
-    </row>
-    <row r="41" ht="17" customHeight="1">
-      <c r="A41" s="288" t="inlineStr">
+      <c r="B46" s="285" t="n"/>
+      <c r="C46" s="308" t="n"/>
+      <c r="D46" s="334" t="n"/>
+      <c r="E46" s="334" t="n"/>
+      <c r="F46" s="334" t="n"/>
+      <c r="G46" s="334" t="n"/>
+      <c r="H46" s="334" t="n"/>
+      <c r="I46" s="334" t="n"/>
+      <c r="J46" s="334" t="n"/>
+      <c r="K46" s="334" t="n"/>
+      <c r="L46" s="333" t="n"/>
+      <c r="M46" s="308" t="n"/>
+      <c r="N46" s="334" t="n"/>
+      <c r="O46" s="334" t="n"/>
+      <c r="P46" s="334" t="n"/>
+      <c r="Q46" s="334" t="n"/>
+      <c r="R46" s="334" t="n"/>
+      <c r="S46" s="334" t="n"/>
+      <c r="T46" s="334" t="n"/>
+      <c r="U46" s="334" t="n"/>
+      <c r="V46" s="334" t="n"/>
+      <c r="W46" s="334" t="n"/>
+      <c r="X46" s="333" t="n"/>
+      <c r="Y46" s="308" t="n"/>
+      <c r="Z46" s="334" t="n"/>
+      <c r="AA46" s="334" t="n"/>
+      <c r="AB46" s="334" t="n"/>
+      <c r="AC46" s="333" t="n"/>
+      <c r="AD46" s="308" t="n"/>
+      <c r="AE46" s="334" t="n"/>
+      <c r="AF46" s="334" t="n"/>
+      <c r="AG46" s="334" t="n"/>
+      <c r="AH46" s="333" t="n"/>
+      <c r="AI46" s="308" t="n"/>
+      <c r="AJ46" s="334" t="n"/>
+      <c r="AK46" s="333" t="n"/>
+      <c r="AL46" s="308" t="n"/>
+      <c r="AM46" s="334" t="n"/>
+      <c r="AN46" s="333" t="n"/>
+    </row>
+    <row r="47" ht="24" customHeight="1">
+      <c r="A47" s="25" t="n"/>
+    </row>
+    <row r="48" hidden="1" outlineLevel="1">
+      <c r="A48" s="288" t="inlineStr">
         <is>
           <t>5.  APPROVAL / SIGN-OFF</t>
         </is>
       </c>
-      <c r="B41" s="289" t="n"/>
-      <c r="C41" s="289" t="n"/>
-      <c r="D41" s="289" t="n"/>
-      <c r="E41" s="289" t="n"/>
-      <c r="F41" s="289" t="n"/>
-      <c r="G41" s="289" t="n"/>
-      <c r="H41" s="289" t="n"/>
-      <c r="I41" s="289" t="n"/>
-      <c r="J41" s="289" t="n"/>
-      <c r="K41" s="289" t="n"/>
-      <c r="L41" s="289" t="n"/>
-      <c r="M41" s="289" t="n"/>
-      <c r="N41" s="289" t="n"/>
-      <c r="O41" s="289" t="n"/>
-      <c r="P41" s="289" t="n"/>
-      <c r="Q41" s="289" t="n"/>
-      <c r="R41" s="289" t="n"/>
-      <c r="S41" s="289" t="n"/>
-      <c r="T41" s="289" t="n"/>
-      <c r="U41" s="289" t="n"/>
-      <c r="V41" s="289" t="n"/>
-      <c r="W41" s="289" t="n"/>
-      <c r="X41" s="289" t="n"/>
-      <c r="Y41" s="289" t="n"/>
-      <c r="Z41" s="289" t="n"/>
-      <c r="AA41" s="289" t="n"/>
-      <c r="AB41" s="289" t="n"/>
-      <c r="AC41" s="289" t="n"/>
-      <c r="AD41" s="289" t="n"/>
-      <c r="AE41" s="289" t="n"/>
-      <c r="AF41" s="289" t="n"/>
-      <c r="AG41" s="289" t="n"/>
-      <c r="AH41" s="289" t="n"/>
-      <c r="AI41" s="289" t="n"/>
-      <c r="AJ41" s="289" t="n"/>
-      <c r="AK41" s="289" t="n"/>
-      <c r="AL41" s="289" t="n"/>
-      <c r="AM41" s="289" t="n"/>
-      <c r="AN41" s="290" t="n"/>
-    </row>
-    <row r="42" ht="17" customHeight="1">
-      <c r="A42" s="320" t="inlineStr">
+      <c r="B48" s="289" t="n"/>
+      <c r="C48" s="289" t="n"/>
+      <c r="D48" s="289" t="n"/>
+      <c r="E48" s="289" t="n"/>
+      <c r="F48" s="289" t="n"/>
+      <c r="G48" s="289" t="n"/>
+      <c r="H48" s="289" t="n"/>
+      <c r="I48" s="289" t="n"/>
+      <c r="J48" s="289" t="n"/>
+      <c r="K48" s="289" t="n"/>
+      <c r="L48" s="289" t="n"/>
+      <c r="M48" s="289" t="n"/>
+      <c r="N48" s="289" t="n"/>
+      <c r="O48" s="289" t="n"/>
+      <c r="P48" s="289" t="n"/>
+      <c r="Q48" s="289" t="n"/>
+      <c r="R48" s="289" t="n"/>
+      <c r="S48" s="289" t="n"/>
+      <c r="T48" s="289" t="n"/>
+      <c r="U48" s="289" t="n"/>
+      <c r="V48" s="289" t="n"/>
+      <c r="W48" s="289" t="n"/>
+      <c r="X48" s="289" t="n"/>
+      <c r="Y48" s="289" t="n"/>
+      <c r="Z48" s="289" t="n"/>
+      <c r="AA48" s="289" t="n"/>
+      <c r="AB48" s="289" t="n"/>
+      <c r="AC48" s="289" t="n"/>
+      <c r="AD48" s="289" t="n"/>
+      <c r="AE48" s="289" t="n"/>
+      <c r="AF48" s="289" t="n"/>
+      <c r="AG48" s="289" t="n"/>
+      <c r="AH48" s="289" t="n"/>
+      <c r="AI48" s="289" t="n"/>
+      <c r="AJ48" s="289" t="n"/>
+      <c r="AK48" s="289" t="n"/>
+      <c r="AL48" s="289" t="n"/>
+      <c r="AM48" s="289" t="n"/>
+      <c r="AN48" s="290" t="n"/>
+    </row>
+    <row r="49" hidden="1" outlineLevel="1">
+      <c r="A49" s="320" t="inlineStr">
         <is>
           <t>Prepared by</t>
         </is>
       </c>
-      <c r="B42" s="289" t="n"/>
-      <c r="C42" s="289" t="n"/>
-      <c r="D42" s="289" t="n"/>
-      <c r="E42" s="289" t="n"/>
-      <c r="F42" s="289" t="n"/>
-      <c r="G42" s="289" t="n"/>
-      <c r="H42" s="289" t="n"/>
-      <c r="I42" s="289" t="n"/>
-      <c r="J42" s="289" t="n"/>
-      <c r="K42" s="289" t="n"/>
-      <c r="L42" s="289" t="n"/>
-      <c r="M42" s="289" t="n"/>
-      <c r="N42" s="321" t="inlineStr">
+      <c r="B49" s="289" t="n"/>
+      <c r="C49" s="289" t="n"/>
+      <c r="D49" s="289" t="n"/>
+      <c r="E49" s="289" t="n"/>
+      <c r="F49" s="289" t="n"/>
+      <c r="G49" s="289" t="n"/>
+      <c r="H49" s="289" t="n"/>
+      <c r="I49" s="289" t="n"/>
+      <c r="J49" s="289" t="n"/>
+      <c r="K49" s="289" t="n"/>
+      <c r="L49" s="289" t="n"/>
+      <c r="M49" s="289" t="n"/>
+      <c r="N49" s="321" t="inlineStr">
         <is>
           <t>Reviewed by</t>
         </is>
       </c>
-      <c r="O42" s="289" t="n"/>
-      <c r="P42" s="289" t="n"/>
-      <c r="Q42" s="289" t="n"/>
-      <c r="R42" s="289" t="n"/>
-      <c r="S42" s="289" t="n"/>
-      <c r="T42" s="289" t="n"/>
-      <c r="U42" s="289" t="n"/>
-      <c r="V42" s="289" t="n"/>
-      <c r="W42" s="289" t="n"/>
-      <c r="X42" s="289" t="n"/>
-      <c r="Y42" s="289" t="n"/>
-      <c r="Z42" s="289" t="n"/>
-      <c r="AA42" s="322" t="inlineStr">
+      <c r="O49" s="289" t="n"/>
+      <c r="P49" s="289" t="n"/>
+      <c r="Q49" s="289" t="n"/>
+      <c r="R49" s="289" t="n"/>
+      <c r="S49" s="289" t="n"/>
+      <c r="T49" s="289" t="n"/>
+      <c r="U49" s="289" t="n"/>
+      <c r="V49" s="289" t="n"/>
+      <c r="W49" s="289" t="n"/>
+      <c r="X49" s="289" t="n"/>
+      <c r="Y49" s="289" t="n"/>
+      <c r="Z49" s="289" t="n"/>
+      <c r="AA49" s="322" t="inlineStr">
         <is>
           <t>Approved by</t>
         </is>
       </c>
-      <c r="AB42" s="289" t="n"/>
-      <c r="AC42" s="289" t="n"/>
-      <c r="AD42" s="289" t="n"/>
-      <c r="AE42" s="289" t="n"/>
-      <c r="AF42" s="289" t="n"/>
-      <c r="AG42" s="289" t="n"/>
-      <c r="AH42" s="289" t="n"/>
-      <c r="AI42" s="289" t="n"/>
-      <c r="AJ42" s="289" t="n"/>
-      <c r="AK42" s="289" t="n"/>
-      <c r="AL42" s="289" t="n"/>
-      <c r="AM42" s="289" t="n"/>
-      <c r="AN42" s="290" t="n"/>
-    </row>
-    <row r="43" ht="26" customHeight="1">
-      <c r="A43" s="323" t="inlineStr">
+      <c r="AB49" s="289" t="n"/>
+      <c r="AC49" s="289" t="n"/>
+      <c r="AD49" s="289" t="n"/>
+      <c r="AE49" s="289" t="n"/>
+      <c r="AF49" s="289" t="n"/>
+      <c r="AG49" s="289" t="n"/>
+      <c r="AH49" s="289" t="n"/>
+      <c r="AI49" s="289" t="n"/>
+      <c r="AJ49" s="289" t="n"/>
+      <c r="AK49" s="289" t="n"/>
+      <c r="AL49" s="289" t="n"/>
+      <c r="AM49" s="289" t="n"/>
+      <c r="AN49" s="290" t="n"/>
+    </row>
+    <row r="50" hidden="1" outlineLevel="1">
+      <c r="A50" s="323" t="inlineStr">
         <is>
           <t>Name  /  Signature  /  Date</t>
         </is>
       </c>
-      <c r="B43" s="268" t="n"/>
-      <c r="C43" s="268" t="n"/>
-      <c r="D43" s="268" t="n"/>
-      <c r="E43" s="268" t="n"/>
-      <c r="F43" s="268" t="n"/>
-      <c r="G43" s="268" t="n"/>
-      <c r="H43" s="268" t="n"/>
-      <c r="I43" s="268" t="n"/>
-      <c r="J43" s="268" t="n"/>
-      <c r="K43" s="268" t="n"/>
-      <c r="L43" s="268" t="n"/>
-      <c r="M43" s="324" t="n"/>
-      <c r="N43" s="323" t="inlineStr">
+      <c r="B50" s="268" t="n"/>
+      <c r="C50" s="268" t="n"/>
+      <c r="D50" s="268" t="n"/>
+      <c r="E50" s="268" t="n"/>
+      <c r="F50" s="268" t="n"/>
+      <c r="G50" s="268" t="n"/>
+      <c r="H50" s="268" t="n"/>
+      <c r="I50" s="268" t="n"/>
+      <c r="J50" s="268" t="n"/>
+      <c r="K50" s="268" t="n"/>
+      <c r="L50" s="268" t="n"/>
+      <c r="M50" s="324" t="n"/>
+      <c r="N50" s="323" t="inlineStr">
         <is>
           <t>Name  /  Signature  /  Date</t>
         </is>
       </c>
-      <c r="O43" s="268" t="n"/>
-      <c r="P43" s="268" t="n"/>
-      <c r="Q43" s="268" t="n"/>
-      <c r="R43" s="268" t="n"/>
-      <c r="S43" s="268" t="n"/>
-      <c r="T43" s="268" t="n"/>
-      <c r="U43" s="268" t="n"/>
-      <c r="V43" s="268" t="n"/>
-      <c r="W43" s="268" t="n"/>
-      <c r="X43" s="268" t="n"/>
-      <c r="Y43" s="268" t="n"/>
-      <c r="Z43" s="324" t="n"/>
-      <c r="AA43" s="323" t="inlineStr">
+      <c r="O50" s="268" t="n"/>
+      <c r="P50" s="268" t="n"/>
+      <c r="Q50" s="268" t="n"/>
+      <c r="R50" s="268" t="n"/>
+      <c r="S50" s="268" t="n"/>
+      <c r="T50" s="268" t="n"/>
+      <c r="U50" s="268" t="n"/>
+      <c r="V50" s="268" t="n"/>
+      <c r="W50" s="268" t="n"/>
+      <c r="X50" s="268" t="n"/>
+      <c r="Y50" s="268" t="n"/>
+      <c r="Z50" s="324" t="n"/>
+      <c r="AA50" s="323" t="inlineStr">
         <is>
           <t>Name  /  Signature  /  Date</t>
         </is>
       </c>
-      <c r="AB43" s="268" t="n"/>
-      <c r="AC43" s="268" t="n"/>
-      <c r="AD43" s="268" t="n"/>
-      <c r="AE43" s="268" t="n"/>
-      <c r="AF43" s="268" t="n"/>
-      <c r="AG43" s="268" t="n"/>
-      <c r="AH43" s="268" t="n"/>
-      <c r="AI43" s="268" t="n"/>
-      <c r="AJ43" s="268" t="n"/>
-      <c r="AK43" s="268" t="n"/>
-      <c r="AL43" s="268" t="n"/>
-      <c r="AM43" s="268" t="n"/>
-      <c r="AN43" s="324" t="n"/>
-    </row>
-    <row r="44" ht="26" customHeight="1">
-      <c r="A44" s="275" t="n"/>
-      <c r="M44" s="325" t="n"/>
-      <c r="N44" s="275" t="n"/>
-      <c r="Z44" s="325" t="n"/>
-      <c r="AA44" s="275" t="n"/>
-      <c r="AN44" s="325" t="n"/>
-    </row>
-    <row r="45" ht="26" customHeight="1">
-      <c r="A45" s="282" t="n"/>
-      <c r="B45" s="283" t="n"/>
-      <c r="C45" s="283" t="n"/>
-      <c r="D45" s="283" t="n"/>
-      <c r="E45" s="283" t="n"/>
-      <c r="F45" s="283" t="n"/>
-      <c r="G45" s="283" t="n"/>
-      <c r="H45" s="283" t="n"/>
-      <c r="I45" s="283" t="n"/>
-      <c r="J45" s="283" t="n"/>
-      <c r="K45" s="283" t="n"/>
-      <c r="L45" s="283" t="n"/>
-      <c r="M45" s="287" t="n"/>
-      <c r="N45" s="282" t="n"/>
-      <c r="O45" s="283" t="n"/>
-      <c r="P45" s="283" t="n"/>
-      <c r="Q45" s="283" t="n"/>
-      <c r="R45" s="283" t="n"/>
-      <c r="S45" s="283" t="n"/>
-      <c r="T45" s="283" t="n"/>
-      <c r="U45" s="283" t="n"/>
-      <c r="V45" s="283" t="n"/>
-      <c r="W45" s="283" t="n"/>
-      <c r="X45" s="283" t="n"/>
-      <c r="Y45" s="283" t="n"/>
-      <c r="Z45" s="287" t="n"/>
-      <c r="AA45" s="282" t="n"/>
-      <c r="AB45" s="283" t="n"/>
-      <c r="AC45" s="283" t="n"/>
-      <c r="AD45" s="283" t="n"/>
-      <c r="AE45" s="283" t="n"/>
-      <c r="AF45" s="283" t="n"/>
-      <c r="AG45" s="283" t="n"/>
-      <c r="AH45" s="283" t="n"/>
-      <c r="AI45" s="283" t="n"/>
-      <c r="AJ45" s="283" t="n"/>
-      <c r="AK45" s="283" t="n"/>
-      <c r="AL45" s="283" t="n"/>
-      <c r="AM45" s="283" t="n"/>
-      <c r="AN45" s="287" t="n"/>
-    </row>
-    <row r="46" ht="4" customHeight="1">
-      <c r="A46" s="25" t="n"/>
-    </row>
-    <row r="47" ht="24" customHeight="1">
-      <c r="A47" s="326" t="inlineStr">
-        <is>
-          <t>NOTICE  —  Enter data only in designated white input cells. Do not add, delete or resize columns/rows. File naming: FRM-202_[RECORDID]_[YYYYMMDD].xlsx | Controlled source sets: Epicor / M365 / approved ANNEX references only.</t>
-        </is>
-      </c>
-      <c r="B47" s="289" t="n"/>
-      <c r="C47" s="289" t="n"/>
-      <c r="D47" s="289" t="n"/>
-      <c r="E47" s="289" t="n"/>
-      <c r="F47" s="289" t="n"/>
-      <c r="G47" s="289" t="n"/>
-      <c r="H47" s="289" t="n"/>
-      <c r="I47" s="289" t="n"/>
-      <c r="J47" s="289" t="n"/>
-      <c r="K47" s="289" t="n"/>
-      <c r="L47" s="289" t="n"/>
-      <c r="M47" s="289" t="n"/>
-      <c r="N47" s="289" t="n"/>
-      <c r="O47" s="289" t="n"/>
-      <c r="P47" s="289" t="n"/>
-      <c r="Q47" s="289" t="n"/>
-      <c r="R47" s="289" t="n"/>
-      <c r="S47" s="289" t="n"/>
-      <c r="T47" s="289" t="n"/>
-      <c r="U47" s="289" t="n"/>
-      <c r="V47" s="289" t="n"/>
-      <c r="W47" s="289" t="n"/>
-      <c r="X47" s="289" t="n"/>
-      <c r="Y47" s="289" t="n"/>
-      <c r="Z47" s="289" t="n"/>
-      <c r="AA47" s="289" t="n"/>
-      <c r="AB47" s="289" t="n"/>
-      <c r="AC47" s="289" t="n"/>
-      <c r="AD47" s="289" t="n"/>
-      <c r="AE47" s="289" t="n"/>
-      <c r="AF47" s="289" t="n"/>
-      <c r="AG47" s="289" t="n"/>
-      <c r="AH47" s="289" t="n"/>
-      <c r="AI47" s="289" t="n"/>
-      <c r="AJ47" s="289" t="n"/>
-      <c r="AK47" s="289" t="n"/>
-      <c r="AL47" s="289" t="n"/>
-      <c r="AM47" s="289" t="n"/>
-      <c r="AN47" s="290" t="n"/>
-    </row>
-    <row r="48" hidden="1" outlineLevel="1"/>
-    <row r="49" hidden="1" outlineLevel="1"/>
-    <row r="50" hidden="1" outlineLevel="1"/>
-    <row r="51" hidden="1" outlineLevel="1"/>
-    <row r="52" hidden="1" outlineLevel="1"/>
-    <row r="53" hidden="1" outlineLevel="1"/>
-    <row r="54" hidden="1" outlineLevel="1"/>
+      <c r="AB50" s="268" t="n"/>
+      <c r="AC50" s="268" t="n"/>
+      <c r="AD50" s="268" t="n"/>
+      <c r="AE50" s="268" t="n"/>
+      <c r="AF50" s="268" t="n"/>
+      <c r="AG50" s="268" t="n"/>
+      <c r="AH50" s="268" t="n"/>
+      <c r="AI50" s="268" t="n"/>
+      <c r="AJ50" s="268" t="n"/>
+      <c r="AK50" s="268" t="n"/>
+      <c r="AL50" s="268" t="n"/>
+      <c r="AM50" s="268" t="n"/>
+      <c r="AN50" s="324" t="n"/>
+    </row>
+    <row r="51" hidden="1" outlineLevel="1">
+      <c r="A51" s="275" t="n"/>
+      <c r="M51" s="325" t="n"/>
+      <c r="N51" s="275" t="n"/>
+      <c r="Z51" s="325" t="n"/>
+      <c r="AA51" s="275" t="n"/>
+      <c r="AN51" s="325" t="n"/>
+    </row>
+    <row r="52" hidden="1" outlineLevel="1">
+      <c r="A52" s="282" t="n"/>
+      <c r="B52" s="283" t="n"/>
+      <c r="C52" s="283" t="n"/>
+      <c r="D52" s="283" t="n"/>
+      <c r="E52" s="283" t="n"/>
+      <c r="F52" s="283" t="n"/>
+      <c r="G52" s="283" t="n"/>
+      <c r="H52" s="283" t="n"/>
+      <c r="I52" s="283" t="n"/>
+      <c r="J52" s="283" t="n"/>
+      <c r="K52" s="283" t="n"/>
+      <c r="L52" s="283" t="n"/>
+      <c r="M52" s="287" t="n"/>
+      <c r="N52" s="282" t="n"/>
+      <c r="O52" s="283" t="n"/>
+      <c r="P52" s="283" t="n"/>
+      <c r="Q52" s="283" t="n"/>
+      <c r="R52" s="283" t="n"/>
+      <c r="S52" s="283" t="n"/>
+      <c r="T52" s="283" t="n"/>
+      <c r="U52" s="283" t="n"/>
+      <c r="V52" s="283" t="n"/>
+      <c r="W52" s="283" t="n"/>
+      <c r="X52" s="283" t="n"/>
+      <c r="Y52" s="283" t="n"/>
+      <c r="Z52" s="287" t="n"/>
+      <c r="AA52" s="282" t="n"/>
+      <c r="AB52" s="283" t="n"/>
+      <c r="AC52" s="283" t="n"/>
+      <c r="AD52" s="283" t="n"/>
+      <c r="AE52" s="283" t="n"/>
+      <c r="AF52" s="283" t="n"/>
+      <c r="AG52" s="283" t="n"/>
+      <c r="AH52" s="283" t="n"/>
+      <c r="AI52" s="283" t="n"/>
+      <c r="AJ52" s="283" t="n"/>
+      <c r="AK52" s="283" t="n"/>
+      <c r="AL52" s="283" t="n"/>
+      <c r="AM52" s="283" t="n"/>
+      <c r="AN52" s="287" t="n"/>
+    </row>
+    <row r="53" hidden="1" outlineLevel="1">
+      <c r="A53" s="25" t="n"/>
+    </row>
+    <row r="54" hidden="1" outlineLevel="1">
+      <c r="A54" s="326" t="inlineStr">
+        <is>
+          <t>NOTICE  -  Enter data only in designated white input cells. Do not add, delete or resize columns/rows. File naming: FRM-202_{Customer}_{PO}.xlsx. Ref: SOP-201 / WI-201, WI-202, WI-203. Retain 10 years per QMS retention schedule.</t>
+        </is>
+      </c>
+      <c r="B54" s="289" t="n"/>
+      <c r="C54" s="289" t="n"/>
+      <c r="D54" s="289" t="n"/>
+      <c r="E54" s="289" t="n"/>
+      <c r="F54" s="289" t="n"/>
+      <c r="G54" s="289" t="n"/>
+      <c r="H54" s="289" t="n"/>
+      <c r="I54" s="289" t="n"/>
+      <c r="J54" s="289" t="n"/>
+      <c r="K54" s="289" t="n"/>
+      <c r="L54" s="289" t="n"/>
+      <c r="M54" s="289" t="n"/>
+      <c r="N54" s="289" t="n"/>
+      <c r="O54" s="289" t="n"/>
+      <c r="P54" s="289" t="n"/>
+      <c r="Q54" s="289" t="n"/>
+      <c r="R54" s="289" t="n"/>
+      <c r="S54" s="289" t="n"/>
+      <c r="T54" s="289" t="n"/>
+      <c r="U54" s="289" t="n"/>
+      <c r="V54" s="289" t="n"/>
+      <c r="W54" s="289" t="n"/>
+      <c r="X54" s="289" t="n"/>
+      <c r="Y54" s="289" t="n"/>
+      <c r="Z54" s="289" t="n"/>
+      <c r="AA54" s="289" t="n"/>
+      <c r="AB54" s="289" t="n"/>
+      <c r="AC54" s="289" t="n"/>
+      <c r="AD54" s="289" t="n"/>
+      <c r="AE54" s="289" t="n"/>
+      <c r="AF54" s="289" t="n"/>
+      <c r="AG54" s="289" t="n"/>
+      <c r="AH54" s="289" t="n"/>
+      <c r="AI54" s="289" t="n"/>
+      <c r="AJ54" s="289" t="n"/>
+      <c r="AK54" s="289" t="n"/>
+      <c r="AL54" s="289" t="n"/>
+      <c r="AM54" s="289" t="n"/>
+      <c r="AN54" s="290" t="n"/>
+    </row>
     <row r="55" hidden="1" outlineLevel="1"/>
     <row r="56" hidden="1" outlineLevel="1"/>
     <row r="57" hidden="1" outlineLevel="1"/>
@@ -7530,7 +7836,7 @@
     <row r="199" hidden="1" outlineLevel="1"/>
     <row r="200" hidden="1" outlineLevel="1"/>
   </sheetData>
-  <mergeCells count="187">
+  <mergeCells count="207">
     <mergeCell ref="AM26:AN26"/>
     <mergeCell ref="A17:G17"/>
     <mergeCell ref="AF23:AI23"/>
@@ -7543,16 +7849,20 @@
     <mergeCell ref="C21:E21"/>
     <mergeCell ref="A14:AN14"/>
     <mergeCell ref="I4:AD4"/>
+    <mergeCell ref="AJ34:AL34"/>
     <mergeCell ref="AD35:AH35"/>
     <mergeCell ref="AF22:AI22"/>
     <mergeCell ref="A9:G9"/>
     <mergeCell ref="I1:AD3"/>
     <mergeCell ref="AE4:AH4"/>
+    <mergeCell ref="AF36:AI36"/>
     <mergeCell ref="C23:E23"/>
     <mergeCell ref="U9:AA9"/>
     <mergeCell ref="AD34:AH34"/>
+    <mergeCell ref="AJ36:AL36"/>
     <mergeCell ref="AM24:AN24"/>
     <mergeCell ref="C34:L34"/>
+    <mergeCell ref="AF34:AI34"/>
     <mergeCell ref="T22:AE22"/>
     <mergeCell ref="AL39:AN39"/>
     <mergeCell ref="A27:B27"/>
@@ -7561,6 +7871,7 @@
     <mergeCell ref="A40:AN40"/>
     <mergeCell ref="AJ29:AL29"/>
     <mergeCell ref="AD36:AH36"/>
+    <mergeCell ref="T34:AE34"/>
     <mergeCell ref="T28:AE28"/>
     <mergeCell ref="H9:T9"/>
     <mergeCell ref="AJ22:AL22"/>
@@ -7570,6 +7881,7 @@
     <mergeCell ref="F28:S28"/>
     <mergeCell ref="T30:AE30"/>
     <mergeCell ref="A35:B35"/>
+    <mergeCell ref="A37:G37"/>
     <mergeCell ref="A6:AN6"/>
     <mergeCell ref="AJ21:AL21"/>
     <mergeCell ref="AM25:AN25"/>
@@ -7585,11 +7897,13 @@
     <mergeCell ref="U18:AA18"/>
     <mergeCell ref="C39:L39"/>
     <mergeCell ref="A8:G8"/>
+    <mergeCell ref="AB38:AN38"/>
     <mergeCell ref="AF26:AI26"/>
     <mergeCell ref="C22:E22"/>
     <mergeCell ref="I5:AD5"/>
     <mergeCell ref="U8:AA8"/>
     <mergeCell ref="AB8:AN8"/>
+    <mergeCell ref="AF35:AI35"/>
     <mergeCell ref="AD38:AH38"/>
     <mergeCell ref="A47:AN47"/>
     <mergeCell ref="AM28:AN28"/>
@@ -7613,7 +7927,9 @@
     <mergeCell ref="AJ26:AL26"/>
     <mergeCell ref="A13:AN13"/>
     <mergeCell ref="AF24:AI24"/>
+    <mergeCell ref="AJ35:AL35"/>
     <mergeCell ref="AI3:AN3"/>
+    <mergeCell ref="F36:S36"/>
     <mergeCell ref="AL35:AN35"/>
     <mergeCell ref="H10:T10"/>
     <mergeCell ref="A26:B26"/>
@@ -7626,6 +7942,7 @@
     <mergeCell ref="F22:S22"/>
     <mergeCell ref="C24:E24"/>
     <mergeCell ref="AF25:AI25"/>
+    <mergeCell ref="U37:AA37"/>
     <mergeCell ref="A7:AN7"/>
     <mergeCell ref="A12:G12"/>
     <mergeCell ref="H17:T17"/>
@@ -7641,12 +7958,14 @@
     <mergeCell ref="A34:B34"/>
     <mergeCell ref="F29:S29"/>
     <mergeCell ref="AD39:AH39"/>
+    <mergeCell ref="H37:T37"/>
     <mergeCell ref="AI36:AK36"/>
     <mergeCell ref="AL37:AN37"/>
     <mergeCell ref="AF31:AI31"/>
     <mergeCell ref="A33:AN33"/>
     <mergeCell ref="H12:T12"/>
     <mergeCell ref="A36:B36"/>
+    <mergeCell ref="A38:G38"/>
     <mergeCell ref="AM22:AN22"/>
     <mergeCell ref="T21:AE21"/>
     <mergeCell ref="AF28:AI28"/>
@@ -7658,13 +7977,16 @@
     <mergeCell ref="A19:AN19"/>
     <mergeCell ref="T23:AE23"/>
     <mergeCell ref="A1:H5"/>
+    <mergeCell ref="H38:T38"/>
     <mergeCell ref="F26:S26"/>
     <mergeCell ref="A21:B21"/>
     <mergeCell ref="C28:E28"/>
     <mergeCell ref="AI2:AN2"/>
+    <mergeCell ref="F35:S35"/>
     <mergeCell ref="AE3:AH3"/>
     <mergeCell ref="T27:AE27"/>
     <mergeCell ref="A16:G16"/>
+    <mergeCell ref="T36:AE36"/>
     <mergeCell ref="U17:AA17"/>
     <mergeCell ref="A23:B23"/>
     <mergeCell ref="C30:E30"/>
@@ -7688,10 +8010,13 @@
     <mergeCell ref="A24:B24"/>
     <mergeCell ref="Y38:AC38"/>
     <mergeCell ref="AJ28:AL28"/>
+    <mergeCell ref="F34:S34"/>
     <mergeCell ref="AI4:AN4"/>
     <mergeCell ref="F25:S25"/>
     <mergeCell ref="AI35:AK35"/>
+    <mergeCell ref="U38:AA38"/>
     <mergeCell ref="AJ30:AL30"/>
+    <mergeCell ref="AB37:AN37"/>
     <mergeCell ref="C27:E27"/>
     <mergeCell ref="F30:S30"/>
     <mergeCell ref="A25:B25"/>
@@ -7717,9 +8042,43 @@
     <mergeCell ref="C29:E29"/>
     <mergeCell ref="AA42:AN42"/>
     <mergeCell ref="A31:B31"/>
+    <mergeCell ref="T35:AE35"/>
     <mergeCell ref="H16:T16"/>
   </mergeCells>
-  <dataValidations count="36">
+  <conditionalFormatting sqref="AF22:AI36">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"FAIL"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
+      <formula>"HOLD"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="2">
+      <formula>"PASS"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AB15:AN15">
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="0">
+      <formula>"FAIL"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="5" operator="equal" dxfId="1">
+      <formula>"HOLD"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="6" operator="equal" dxfId="2">
+      <formula>"PASS"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AB18:AN18">
+    <cfRule type="cellIs" priority="7" operator="equal" dxfId="1">
+      <formula>"OPEN"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="8" operator="equal" dxfId="2">
+      <formula>"CLOSED"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="9" operator="equal" dxfId="3">
+      <formula>"IN PROGRESS"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="41">
     <dataValidation sqref="AF22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Use controlled value from VAL_RESULT_CORE." prompt="Select from VAL_RESULT_CORE." type="list">
       <formula1>=VAL_RESULT_CORE</formula1>
     </dataValidation>
@@ -7828,6 +8187,21 @@
     <dataValidation sqref="AB18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Use controlled value from VAL_STATUS_CORE." prompt="Select from VAL_STATUS_CORE." type="list">
       <formula1>=VAL_STATUS_CORE</formula1>
     </dataValidation>
+    <dataValidation sqref="AF32" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid" error="Select PASS, HOLD, FAIL, or NA." type="list">
+      <formula1>=VAL_RESULT_CORE</formula1>
+    </dataValidation>
+    <dataValidation sqref="AF33" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid" error="Select PASS, HOLD, FAIL, or NA." type="list">
+      <formula1>=VAL_RESULT_CORE</formula1>
+    </dataValidation>
+    <dataValidation sqref="AF34" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid" error="Select PASS, HOLD, FAIL, or NA." type="list">
+      <formula1>=VAL_RESULT_CORE</formula1>
+    </dataValidation>
+    <dataValidation sqref="AF35" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid" error="Select PASS, HOLD, FAIL, or NA." type="list">
+      <formula1>=VAL_RESULT_CORE</formula1>
+    </dataValidation>
+    <dataValidation sqref="AF36" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid" error="Select PASS, HOLD, FAIL, or NA." type="list">
+      <formula1>=VAL_RESULT_CORE</formula1>
+    </dataValidation>
   </dataValidations>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.197" right="0.197" top="0.197" bottom="0.197" header="0.1" footer="0.1"/>
@@ -7851,7 +8225,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -7882,6 +8256,21 @@
           <t>VAL_RISK_LEVEL_CORE</t>
         </is>
       </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>VAL_YES_NO</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>VAL_DISCOVERY_STAGE</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>VAL_CK_CATEGORY</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -7904,6 +8293,21 @@
           <t>LOW</t>
         </is>
       </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>INCOMING</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>COM</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -7926,6 +8330,21 @@
           <t>MEDIUM</t>
         </is>
       </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>SETUP</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>TEC</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -7948,6 +8367,21 @@
           <t>HIGH</t>
         </is>
       </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>FIRST PIECE</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>QUA</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -7970,6 +8404,16 @@
           <t>CRITICAL</t>
         </is>
       </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>IN-PROCESS</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>CAP</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="C6" t="inlineStr">
@@ -7977,6 +8421,16 @@
           <t>SUPERSEDED</t>
         </is>
       </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>FINAL INSPECTION</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>CON</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="C7" t="inlineStr">
@@ -7984,9 +8438,41 @@
           <t>VOID</t>
         </is>
       </c>
-    </row>
-    <row r="8" hidden="1"/>
-    <row r="9" hidden="1"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>PACKAGING</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>DOC</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" hidden="1">
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>SHIPPING</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>REL</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" hidden="1">
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>CUSTOMER</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>CNC</t>
+        </is>
+      </c>
+    </row>
     <row r="10" hidden="1"/>
     <row r="11" hidden="1"/>
     <row r="12" hidden="1"/>
@@ -8512,7 +8998,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr autoPageBreaks="0" fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H28"/>
+  <dimension ref="A1:K28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -8563,6 +9049,11 @@
           <t>V0</t>
         </is>
       </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="275" t="n"/>
@@ -8579,6 +9070,11 @@
       <c r="H3" s="350" t="inlineStr">
         <is>
           <t>YYYY-MM-DD</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>2026-03-22</t>
         </is>
       </c>
     </row>
@@ -9193,6 +9689,17 @@
     <mergeCell ref="A9:B9"/>
     <mergeCell ref="G9:H9"/>
   </mergeCells>
+  <conditionalFormatting sqref="G17:G26">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="1">
+      <formula>"OPEN"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="2">
+      <formula>"CLOSED"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="3">
+      <formula>"IN PROGRESS"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="2">
     <dataValidation sqref="D17:D26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Use controlled value from REF_OWNER_PERSON_MASTER." prompt="Select from REF_OWNER_PERSON_MASTER." type="list">
       <formula1>=REF_OWNER_PERSON_MASTER</formula1>
@@ -9577,4 +10084,106 @@
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="45" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="413" t="inlineStr">
+        <is>
+          <t>Rev</t>
+        </is>
+      </c>
+      <c r="B1" s="413" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C1" s="413" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="D1" s="413" t="inlineStr">
+        <is>
+          <t>Author</t>
+        </is>
+      </c>
+      <c r="E1" s="413" t="inlineStr">
+        <is>
+          <t>Approved By</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="414" t="inlineStr">
+        <is>
+          <t>V0</t>
+        </is>
+      </c>
+      <c r="B2" s="414" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="C2" s="414" t="inlineStr">
+        <is>
+          <t>Initial controlled baseline</t>
+        </is>
+      </c>
+      <c r="D2" s="414" t="inlineStr">
+        <is>
+          <t>QMS</t>
+        </is>
+      </c>
+      <c r="E2" s="414" t="inlineStr">
+        <is>
+          <t>General Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="414" t="inlineStr">
+        <is>
+          <t>V1</t>
+        </is>
+      </c>
+      <c r="B3" s="414" t="inlineStr">
+        <is>
+          <t>2026-03-22</t>
+        </is>
+      </c>
+      <c r="C3" s="414" t="inlineStr">
+        <is>
+          <t>Upgrade: CNC fields, cross-form linkage, conditional formatting, parent procedure ref</t>
+        </is>
+      </c>
+      <c r="D3" s="414" t="inlineStr">
+        <is>
+          <t>QMS</t>
+        </is>
+      </c>
+      <c r="E3" s="414" t="inlineStr">
+        <is>
+          <t>General Manager</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>